<commit_message>
scan: seg5 2026-06-22 21:29 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq6_2026-06-22.xlsx
@@ -580,21 +580,21 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>6415</v>
+        <v>6257</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v/>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1222.513716588245</v>
+        <v>1235.76954120663</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>673</v>
+        <v>242.5</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -605,16 +605,16 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>66.98787001935186</v>
+        <v>64.20404645683077</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>27.86728742720888</v>
+        <v>27.52445723015365</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2.354616567675678</v>
+        <v>2.182837363914051</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>1</v>
@@ -623,31 +623,31 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>4.266115137202064</v>
+        <v>0.7893270278889402</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>6257</v>
+        <v>6415</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>矽格</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1215.76954120663</v>
+        <v>1222.513716588245</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>242.5</v>
+        <v>673</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -658,16 +658,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>64.20404645683077</v>
+        <v>66.98787001935186</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>27.52445723015365</v>
+        <v>27.86728742720888</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2.182837363914051</v>
+        <v>2.354616567675678</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>1</v>
@@ -676,11 +676,11 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.7893270278889402</v>
+        <v>4.266115137202064</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -845,21 +845,21 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6435</v>
+        <v>6271</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>大中</t>
+          <t>同欣電</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1165.207620282458</v>
+        <v>1172.986592783368</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>349</v>
+        <v>266.5</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,49 +870,49 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>74.10282340950839</v>
+        <v>64.24358277257826</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>29.06303213575171</v>
+        <v>26.43904771026768</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.2174668720718798</v>
+        <v>3.046049548946924</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>3.341564650546722</v>
+        <v>-0.4858912132232031</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6271</v>
+        <v>6435</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>同欣電</t>
+          <t>大中</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1157.986592783368</v>
+        <v>1165.207620282458</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>266.5</v>
+        <v>349</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,29 +923,29 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>64.24358277257826</v>
+        <v>74.10282340950839</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>26.43904771026768</v>
+        <v>29.06303213575171</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>3.046049548946924</v>
+        <v>0.2174668720718798</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-0.4858912132232031</v>
+        <v>3.341564650546722</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, hist_turn_positive, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1130.605430569954</v>
+        <v>1150.605430569954</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>31.1</v>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1007.519697804113</v>
+        <v>997.5196978041128</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>97.2</v>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>939.7208796610248</v>
+        <v>949.7208796610248</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>38.35</v>
@@ -2488,21 +2488,21 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6451</v>
+        <v>6282</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>訊芯-KY</t>
+          <t>康舒</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>761.0019185940325</v>
+        <v>766.5641204986298</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>617</v>
+        <v>63.9</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>57.33568182600086</v>
+        <v>58.55972708898098</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>32.11931170361538</v>
+        <v>31.38753500682633</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1.15896498985467</v>
+        <v>0.8819779510114427</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-8.482328342727115</v>
+        <v>-0.5085945680500159</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6282</v>
+        <v>6451</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>康舒</t>
+          <t>訊芯-KY</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>756.5641204986298</v>
+        <v>761.0019185940325</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>63.9</v>
+        <v>617</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>58.55972708898098</v>
+        <v>57.33568182600086</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>31.38753500682633</v>
+        <v>32.11931170361538</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.8819779510114427</v>
+        <v>1.15896498985467</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,11 +2584,11 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.5085945680500159</v>
+        <v>-8.482328342727115</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>618.3487641781219</v>
+        <v>608.3487641781219</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>83.09999999999999</v>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>584.3449736615671</v>
+        <v>594.3449736615671</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>134.5</v>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>344.0623419507396</v>
+        <v>329.0623419507396</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>39</v>
@@ -5138,21 +5138,21 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6246</v>
+        <v>6226</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>臺龍</t>
+          <t>光鼎</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>321.2926025667705</v>
+        <v>324.5270205765061</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>15.35</v>
+        <v>12.5</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>46.36685134335679</v>
+        <v>47.95352750956579</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>17.56104647028084</v>
+        <v>13.42941845221206</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.9886562203149321</v>
+        <v>0.6672309565296523</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>2</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0039927306546469</v>
+        <v>-0.0870051656056928</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6230</v>
+        <v>6246</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>尼得科超眾</t>
+          <t>臺龍</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>319.1948903728893</v>
+        <v>321.2926025667705</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>135</v>
+        <v>15.35</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,16 +5216,16 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>45.72777273350233</v>
+        <v>46.36685134335679</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>12.50673783869418</v>
+        <v>17.56104647028084</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.5832158385899915</v>
+        <v>0.9886562203149321</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.2940331175268151</v>
+        <v>-0.0039927306546469</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6226</v>
+        <v>6230</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>光鼎</t>
+          <t>尼得科超眾</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>314.5270205765061</v>
+        <v>319.1948903728893</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>12.5</v>
+        <v>135</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>47.95352750956579</v>
+        <v>45.72777273350233</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>13.42941845221206</v>
+        <v>12.50673783869418</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.6672309565296523</v>
+        <v>0.5832158385899915</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,11 +5287,11 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.0870051656056928</v>
+        <v>0.2940331175268151</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
@@ -5880,21 +5880,21 @@
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6216</v>
+        <v>6176</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>居易</t>
+          <t>瑞儀</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>228.1434890348388</v>
+        <v>228.8480948863965</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>23.3</v>
+        <v>90.2</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>53.2253218148581</v>
+        <v>38.61297861512627</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>18.02621570282329</v>
+        <v>28.60535134726064</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.5575212104461752</v>
+        <v>1.281212761903083</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.09594091132618909</v>
+        <v>-1.001463651668665</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6176</v>
+        <v>6216</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>瑞儀</t>
+          <t>居易</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>218.8480948863965</v>
+        <v>228.1434890348388</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>90.2</v>
+        <v>23.3</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>38.61297861512627</v>
+        <v>53.2253218148581</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>28.60535134726064</v>
+        <v>18.02621570282329</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1.281212761903083</v>
+        <v>0.5575212104461752</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,11 +5976,11 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-1.001463651668665</v>
+        <v>0.09594091132618909</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>

</xml_diff>